<commit_message>
update objective function evaluation
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Academia\Research related\dev\VRP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F5BF56-71D6-40F8-8A8F-0B9812F33C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F04969-69D9-418E-BE12-30B9C6A50C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="3690" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5445" yWindow="4950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VRPTW Benchmarking" sheetId="1" r:id="rId1"/>
@@ -1713,15 +1713,15 @@
         <v>6.0679091434630017E-3</v>
       </c>
       <c r="F65" s="5">
-        <f>4.43/1000</f>
-        <v>4.4299999999999999E-3</v>
+        <f>4.42/1000</f>
+        <v>4.4200000000000003E-3</v>
       </c>
       <c r="G65" s="1">
         <v>2000</v>
       </c>
       <c r="H65" s="6">
         <f>F65 * G65</f>
-        <v>8.86</v>
+        <v>8.84</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
@@ -1742,15 +1742,15 @@
         <v>-2.4680298313238036E-2</v>
       </c>
       <c r="F66" s="4">
-        <f>14.93/1000</f>
-        <v>1.4930000000000001E-2</v>
+        <f>14.74/1000</f>
+        <v>1.474E-2</v>
       </c>
       <c r="G66" s="1">
         <v>2000</v>
       </c>
       <c r="H66" s="6">
         <f t="shared" ref="H66:H70" si="1">F66 * G66</f>
-        <v>29.86</v>
+        <v>29.48</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
@@ -1771,15 +1771,15 @@
         <v>-3.7795947102070571E-6</v>
       </c>
       <c r="F67" s="4">
-        <f>5.92/1000</f>
-        <v>5.9199999999999999E-3</v>
+        <f>5.91/1000</f>
+        <v>5.9100000000000003E-3</v>
       </c>
       <c r="G67" s="1">
         <v>2000</v>
       </c>
       <c r="H67" s="6">
         <f t="shared" si="1"/>
-        <v>11.84</v>
+        <v>11.82</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
@@ -1800,15 +1800,15 @@
         <v>-5.8207624822337323E-6</v>
       </c>
       <c r="F68" s="4">
-        <f>23.85/1000</f>
-        <v>2.3850000000000003E-2</v>
+        <f>23.8/1000</f>
+        <v>2.3800000000000002E-2</v>
       </c>
       <c r="G68" s="1">
         <v>2000</v>
       </c>
       <c r="H68" s="6">
         <f t="shared" si="1"/>
-        <v>47.7</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -1829,15 +1829,15 @@
         <v>7.1676315548516722E-3</v>
       </c>
       <c r="F69" s="4">
-        <f>4.87/1000</f>
-        <v>4.8700000000000002E-3</v>
+        <f>4.88/1000</f>
+        <v>4.8799999999999998E-3</v>
       </c>
       <c r="G69" s="1">
         <v>2000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="1"/>
-        <v>9.74</v>
+        <v>9.76</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -1858,15 +1858,15 @@
         <v>-1.7050732349624509E-2</v>
       </c>
       <c r="F70" s="4">
-        <f>9.01/1000</f>
-        <v>9.0100000000000006E-3</v>
+        <f>14.58/1000</f>
+        <v>1.4579999999999999E-2</v>
       </c>
       <c r="G70" s="1">
         <v>2000</v>
       </c>
       <c r="H70" s="6">
         <f t="shared" si="1"/>
-        <v>18.02</v>
+        <v>29.16</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
add temporal dimension to relatedness
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Academia\Research related\dev\VRP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F04969-69D9-418E-BE12-30B9C6A50C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D9240E-2814-4FD2-B704-5D24527C08CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5445" yWindow="4950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VRPTW Benchmarking" sheetId="1" r:id="rId1"/>
@@ -1706,22 +1706,22 @@
         <v>1645.79</v>
       </c>
       <c r="D65" s="6">
-        <v>1655.7765041892201</v>
+        <v>1671.24036467372</v>
       </c>
       <c r="E65" s="3">
         <f>D65/C65-1</f>
-        <v>6.0679091434630017E-3</v>
+        <v>1.5463919864454168E-2</v>
       </c>
       <c r="F65" s="5">
-        <f>4.42/1000</f>
-        <v>4.4200000000000003E-3</v>
+        <f>5.4/1000</f>
+        <v>5.4000000000000003E-3</v>
       </c>
       <c r="G65" s="1">
         <v>2000</v>
       </c>
       <c r="H65" s="6">
         <f>F65 * G65</f>
-        <v>8.84</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
@@ -1735,22 +1735,22 @@
         <v>1252.3699999999999</v>
       </c>
       <c r="D66" s="24">
-        <v>1221.46113480145</v>
+        <v>1224.5023993416801</v>
       </c>
       <c r="E66" s="3">
         <f t="shared" ref="E66:E70" si="0">D66/C66-1</f>
-        <v>-2.4680298313238036E-2</v>
+        <v>-2.2251890941430874E-2</v>
       </c>
       <c r="F66" s="4">
-        <f>14.74/1000</f>
-        <v>1.474E-2</v>
+        <f>16.66/1000</f>
+        <v>1.6660000000000001E-2</v>
       </c>
       <c r="G66" s="1">
         <v>2000</v>
       </c>
       <c r="H66" s="6">
         <f t="shared" ref="H66:H70" si="1">F66 * G66</f>
-        <v>29.48</v>
+        <v>33.32</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
@@ -1764,22 +1764,22 @@
         <v>828.94</v>
       </c>
       <c r="D67" s="6">
-        <v>828.93686694276096</v>
+        <v>828.93686694277699</v>
       </c>
       <c r="E67" s="3">
         <f t="shared" si="0"/>
-        <v>-3.7795947102070571E-6</v>
+        <v>-3.7795946908891764E-6</v>
       </c>
       <c r="F67" s="4">
-        <f>5.91/1000</f>
-        <v>5.9100000000000003E-3</v>
+        <f>6.55/1000</f>
+        <v>6.5499999999999994E-3</v>
       </c>
       <c r="G67" s="1">
         <v>2000</v>
       </c>
       <c r="H67" s="6">
         <f t="shared" si="1"/>
-        <v>11.82</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
@@ -1793,22 +1793,22 @@
         <v>591.55999999999995</v>
       </c>
       <c r="D68" s="6">
-        <v>591.55655666974599</v>
+        <v>591.55655666806399</v>
       </c>
       <c r="E68" s="3">
         <f t="shared" si="0"/>
-        <v>-5.8207624822337323E-6</v>
+        <v>-5.8207653255148983E-6</v>
       </c>
       <c r="F68" s="4">
-        <f>23.8/1000</f>
-        <v>2.3800000000000002E-2</v>
+        <f>28.24/1000</f>
+        <v>2.8239999999999998E-2</v>
       </c>
       <c r="G68" s="1">
         <v>2000</v>
       </c>
       <c r="H68" s="6">
         <f t="shared" si="1"/>
-        <v>47.6</v>
+        <v>56.48</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -1822,22 +1822,22 @@
         <v>1696.94</v>
       </c>
       <c r="D69" s="6">
-        <v>1709.10304069069</v>
+        <v>1668.3899931731401</v>
       </c>
       <c r="E69" s="3">
         <f t="shared" si="0"/>
-        <v>7.1676315548516722E-3</v>
+        <v>-1.6824405592926084E-2</v>
       </c>
       <c r="F69" s="4">
-        <f>4.88/1000</f>
-        <v>4.8799999999999998E-3</v>
+        <f>5.81/1000</f>
+        <v>5.8099999999999992E-3</v>
       </c>
       <c r="G69" s="1">
         <v>2000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="1"/>
-        <v>9.76</v>
+        <v>11.62</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -1851,22 +1851,22 @@
         <v>1406.91</v>
       </c>
       <c r="D70" s="24">
-        <v>1382.9211541499899</v>
+        <v>1354.4467482727</v>
       </c>
       <c r="E70" s="3">
         <f t="shared" si="0"/>
-        <v>-1.7050732349624509E-2</v>
+        <v>-3.7289699929135556E-2</v>
       </c>
       <c r="F70" s="4">
-        <f>14.58/1000</f>
-        <v>1.4579999999999999E-2</v>
+        <f>17.37/1000</f>
+        <v>1.737E-2</v>
       </c>
       <c r="G70" s="1">
         <v>2000</v>
       </c>
       <c r="H70" s="6">
         <f t="shared" si="1"/>
-        <v>29.16</v>
+        <v>34.74</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
upadte redundant vehicle/route handling
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Academia\Research related\dev\VRP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF76458-9B20-4749-A95E-5C7FD9842AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D9E1FC-41CF-47EF-ABBF-A07A56A0CD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1713,15 +1713,15 @@
         <v>1.5463919864454168E-2</v>
       </c>
       <c r="F65" s="5">
-        <f>4.88/1000</f>
-        <v>4.8799999999999998E-3</v>
+        <f>4.82/1000</f>
+        <v>4.8200000000000005E-3</v>
       </c>
       <c r="G65" s="1">
         <v>2000</v>
       </c>
       <c r="H65" s="6">
         <f>F65 * G65</f>
-        <v>9.76</v>
+        <v>9.64</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
@@ -1742,15 +1742,15 @@
         <v>-2.2251890941430874E-2</v>
       </c>
       <c r="F66" s="4">
-        <f>14.31/1000</f>
-        <v>1.431E-2</v>
+        <f>14.49/1000</f>
+        <v>1.4489999999999999E-2</v>
       </c>
       <c r="G66" s="1">
         <v>2000</v>
       </c>
       <c r="H66" s="6">
         <f t="shared" ref="H66:H70" si="1">F66 * G66</f>
-        <v>28.62</v>
+        <v>28.98</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
@@ -1771,15 +1771,15 @@
         <v>-3.7795946908891764E-6</v>
       </c>
       <c r="F67" s="4">
-        <f>6.1/1000</f>
-        <v>6.0999999999999995E-3</v>
+        <f>6.07/1000</f>
+        <v>6.0699999999999999E-3</v>
       </c>
       <c r="G67" s="1">
         <v>2000</v>
       </c>
       <c r="H67" s="6">
         <f t="shared" si="1"/>
-        <v>12.2</v>
+        <v>12.14</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
@@ -1800,15 +1800,15 @@
         <v>-5.8207653255148983E-6</v>
       </c>
       <c r="F68" s="4">
-        <f>24.84/1000</f>
-        <v>2.4840000000000001E-2</v>
+        <f>24.92/1000</f>
+        <v>2.4920000000000001E-2</v>
       </c>
       <c r="G68" s="1">
         <v>2000</v>
       </c>
       <c r="H68" s="6">
         <f t="shared" si="1"/>
-        <v>49.68</v>
+        <v>49.84</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -1829,15 +1829,15 @@
         <v>-1.6824405592926084E-2</v>
       </c>
       <c r="F69" s="4">
-        <f>5.12/1000</f>
-        <v>5.1200000000000004E-3</v>
+        <f>5.1/1000</f>
+        <v>5.0999999999999995E-3</v>
       </c>
       <c r="G69" s="1">
         <v>2000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="1"/>
-        <v>10.24</v>
+        <v>10.199999999999999</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -1858,15 +1858,15 @@
         <v>-3.7289699929135556E-2</v>
       </c>
       <c r="F70" s="4">
-        <f>15.52/1000</f>
-        <v>1.5519999999999999E-2</v>
+        <f>15.5/1000</f>
+        <v>1.55E-2</v>
       </c>
       <c r="G70" s="1">
         <v>2000</v>
       </c>
       <c r="H70" s="6">
         <f t="shared" si="1"/>
-        <v>31.04</v>
+        <v>31</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
update operations & insertion cost
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Academia\Research related\dev\VRP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC42350-65BE-4F42-A032-770924E9118F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BDF6E20-244C-4D8A-8720-43F00A46FDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-113" yWindow="-113" windowWidth="48309" windowHeight="26546" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1706,22 +1706,22 @@
         <v>1645.79</v>
       </c>
       <c r="D65" s="6">
-        <v>1647.99912450019</v>
+        <v>1643.0888648786899</v>
       </c>
       <c r="E65" s="3">
         <f>D65/C65-1</f>
-        <v>1.34228820213389E-3</v>
+        <v>-1.6412392354492322E-3</v>
       </c>
       <c r="F65" s="5">
-        <f>4.71/1000</f>
-        <v>4.7099999999999998E-3</v>
+        <f>4.79/1000</f>
+        <v>4.79E-3</v>
       </c>
       <c r="G65" s="1">
         <v>2000</v>
       </c>
       <c r="H65" s="6">
         <f>F65 * G65</f>
-        <v>9.42</v>
+        <v>9.58</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
@@ -1735,22 +1735,22 @@
         <v>1252.3699999999999</v>
       </c>
       <c r="D66" s="24">
-        <v>1201.06719688372</v>
+        <v>1196.2386137594799</v>
       </c>
       <c r="E66" s="3">
         <f t="shared" ref="E66:E70" si="0">D66/C66-1</f>
-        <v>-4.0964573661361969E-2</v>
+        <v>-4.4820130025886917E-2</v>
       </c>
       <c r="F66" s="4">
-        <f>13.07/1000</f>
-        <v>1.307E-2</v>
+        <f>12.42/1000</f>
+        <v>1.242E-2</v>
       </c>
       <c r="G66" s="1">
         <v>2000</v>
       </c>
       <c r="H66" s="6">
         <f t="shared" ref="H66:H70" si="1">F66 * G66</f>
-        <v>26.14</v>
+        <v>24.84</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
@@ -1764,22 +1764,22 @@
         <v>828.94</v>
       </c>
       <c r="D67" s="6">
-        <v>828.93686694277699</v>
+        <v>828.93686694224698</v>
       </c>
       <c r="E67" s="3">
         <f t="shared" si="0"/>
-        <v>-3.7795946908891764E-6</v>
+        <v>-3.7795953302666163E-6</v>
       </c>
       <c r="F67" s="4">
-        <f>6.13/1000</f>
-        <v>6.13E-3</v>
+        <f>6.65/1000</f>
+        <v>6.6500000000000005E-3</v>
       </c>
       <c r="G67" s="1">
         <v>2000</v>
       </c>
       <c r="H67" s="6">
         <f t="shared" si="1"/>
-        <v>12.26</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -1793,22 +1793,22 @@
         <v>591.55999999999995</v>
       </c>
       <c r="D68" s="6">
-        <v>591.55655666806399</v>
+        <v>591.55655666872997</v>
       </c>
       <c r="E68" s="3">
         <f t="shared" si="0"/>
-        <v>-5.8207653255148983E-6</v>
+        <v>-5.8207641997487514E-6</v>
       </c>
       <c r="F68" s="4">
-        <f>24.34/1000</f>
-        <v>2.4340000000000001E-2</v>
+        <f>22.92/1000</f>
+        <v>2.2920000000000003E-2</v>
       </c>
       <c r="G68" s="1">
         <v>2000</v>
       </c>
       <c r="H68" s="6">
         <f t="shared" si="1"/>
-        <v>48.68</v>
+        <v>45.84</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -1822,22 +1822,22 @@
         <v>1696.94</v>
       </c>
       <c r="D69" s="6">
-        <v>1678.1751810066401</v>
+        <v>1670.2230616634599</v>
       </c>
       <c r="E69" s="3">
         <f t="shared" si="0"/>
-        <v>-1.1058033279526702E-2</v>
+        <v>-1.57441856144237E-2</v>
       </c>
       <c r="F69" s="4">
-        <f>4.74/1000</f>
-        <v>4.7400000000000003E-3</v>
+        <f>12.69/1000</f>
+        <v>1.269E-2</v>
       </c>
       <c r="G69" s="1">
         <v>2000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="1"/>
-        <v>9.48</v>
+        <v>25.38</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -1851,22 +1851,22 @@
         <v>1406.91</v>
       </c>
       <c r="D70" s="24">
-        <v>1409.21629394568</v>
+        <v>1297.91070367663</v>
       </c>
       <c r="E70" s="3">
         <f t="shared" si="0"/>
-        <v>1.6392618900142875E-3</v>
+        <v>-7.7474249471089163E-2</v>
       </c>
       <c r="F70" s="4">
-        <f>14.85/1000</f>
-        <v>1.485E-2</v>
+        <f>5.25/1000</f>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="G70" s="1">
         <v>2000</v>
       </c>
       <c r="H70" s="6">
         <f t="shared" si="1"/>
-        <v>29.7</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
test for non- time-window instances
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Academia\Research related\dev\VRP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BDF6E20-244C-4D8A-8720-43F00A46FDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F631D79-84C4-4324-A7BE-FCEAED795386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="48309" windowHeight="26546" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="48309" windowHeight="26546" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="VRPTW Benchmarking" sheetId="1" r:id="rId1"/>
+    <sheet name="VRP Benchmarking" sheetId="2" r:id="rId1"/>
+    <sheet name="VRPTW Benchmarking" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="93">
   <si>
     <t>Best known</t>
   </si>
@@ -271,10 +272,49 @@
     <t>x = length(N)</t>
   </si>
   <si>
-    <t>n = ceil(x, digits=-(length(digits(x))-1))</t>
-  </si>
-  <si>
     <t>Vehicle Routing Problem with Time-Windows (VRPTW) Benchmarking</t>
+  </si>
+  <si>
+    <t>Vehicle Routing Problem (VRP) Benchmarking</t>
+  </si>
+  <si>
+    <t>Initializtion</t>
+  </si>
+  <si>
+    <t>:random</t>
+  </si>
+  <si>
+    <t>                    :worstnode!     ,  </t>
+  </si>
+  <si>
+    <t>                    :relatedroute!  ,</t>
+  </si>
+  <si>
+    <t>                    :worstroute!</t>
+  </si>
+  <si>
+    <t>                    :regret2!       ,</t>
+  </si>
+  <si>
+    <t>m-n101-k10</t>
+  </si>
+  <si>
+    <t>tai150a</t>
+  </si>
+  <si>
+    <t>cmt10</t>
+  </si>
+  <si>
+    <t>x-n251-k28</t>
+  </si>
+  <si>
+    <t>x-n303-k21</t>
+  </si>
+  <si>
+    <t>χ   = ALNSParameters(</t>
+  </si>
+  <si>
+    <t>n = max(200, ceil(x, digits=-(length(digits(x))-1)))</t>
   </si>
 </sst>
 </file>
@@ -464,7 +504,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -504,6 +544,16 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -784,6 +834,1549 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EB48D86-1312-4781-AFB7-1DCAC26244E4}">
+  <dimension ref="A1:X274"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15.05" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.05" x14ac:dyDescent="0.3">
+      <c r="A2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="8"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="12"/>
+      <c r="U18" s="12"/>
+      <c r="V18" s="12"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="12"/>
+    </row>
+    <row r="19" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="L19" s="12"/>
+      <c r="W19" s="12"/>
+      <c r="X19" s="12"/>
+    </row>
+    <row r="20" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="L20" s="12"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="12"/>
+    </row>
+    <row r="21" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="L21" s="12"/>
+      <c r="U21" s="12"/>
+      <c r="V21" s="12"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="12"/>
+    </row>
+    <row r="22" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="L22" s="12"/>
+      <c r="U22" s="12"/>
+      <c r="V22" s="12"/>
+      <c r="W22" s="12"/>
+      <c r="X22" s="12"/>
+    </row>
+    <row r="23" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="U23" s="12"/>
+      <c r="V23" s="12"/>
+      <c r="W23" s="12"/>
+      <c r="X23" s="12"/>
+    </row>
+    <row r="24" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="U24" s="12"/>
+      <c r="V24" s="12"/>
+      <c r="W24" s="12"/>
+      <c r="X24" s="12"/>
+    </row>
+    <row r="25" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="U25" s="12"/>
+      <c r="V25" s="12"/>
+      <c r="W25" s="12"/>
+      <c r="X25" s="12"/>
+    </row>
+    <row r="26" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="U26" s="12"/>
+      <c r="V26" s="12"/>
+      <c r="W26" s="12"/>
+      <c r="X26" s="12"/>
+    </row>
+    <row r="27" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="L27" s="12"/>
+      <c r="U27" s="12"/>
+      <c r="V27" s="12"/>
+      <c r="W27" s="12"/>
+      <c r="X27" s="12"/>
+    </row>
+    <row r="28" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="11"/>
+      <c r="L28" s="12"/>
+      <c r="U28" s="12"/>
+      <c r="V28" s="12"/>
+      <c r="W28" s="12"/>
+      <c r="X28" s="12"/>
+    </row>
+    <row r="29" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="11"/>
+      <c r="L29" s="12"/>
+      <c r="U29" s="12"/>
+      <c r="V29" s="12"/>
+      <c r="W29" s="12"/>
+      <c r="X29" s="12"/>
+    </row>
+    <row r="30" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="L30" s="12"/>
+      <c r="U30" s="12"/>
+      <c r="V30" s="12"/>
+      <c r="W30" s="12"/>
+      <c r="X30" s="12"/>
+    </row>
+    <row r="31" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" s="11"/>
+      <c r="L31" s="12"/>
+      <c r="U31" s="12"/>
+      <c r="V31" s="12"/>
+      <c r="W31" s="12"/>
+      <c r="X31" s="12"/>
+    </row>
+    <row r="32" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" s="11"/>
+      <c r="L32" s="12"/>
+      <c r="U32" s="12"/>
+      <c r="V32" s="12"/>
+      <c r="W32" s="12"/>
+      <c r="X32" s="12"/>
+    </row>
+    <row r="33" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33" s="11"/>
+      <c r="L33" s="12"/>
+      <c r="U33" s="12"/>
+      <c r="V33" s="12"/>
+      <c r="W33" s="12"/>
+      <c r="X33" s="12"/>
+    </row>
+    <row r="34" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" s="11"/>
+      <c r="L34" s="12"/>
+      <c r="U34" s="12"/>
+      <c r="V34" s="12"/>
+      <c r="W34" s="12"/>
+      <c r="X34" s="12"/>
+    </row>
+    <row r="35" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="L35" s="12"/>
+      <c r="U35" s="12"/>
+      <c r="V35" s="12"/>
+      <c r="W35" s="12"/>
+      <c r="X35" s="12"/>
+    </row>
+    <row r="36" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="L36" s="12"/>
+      <c r="U36" s="12"/>
+      <c r="V36" s="12"/>
+      <c r="W36" s="12"/>
+      <c r="X36" s="12"/>
+    </row>
+    <row r="37" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="L37" s="12"/>
+      <c r="U37" s="12"/>
+      <c r="V37" s="12"/>
+      <c r="W37" s="12"/>
+      <c r="X37" s="12"/>
+    </row>
+    <row r="38" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" s="11"/>
+      <c r="L38" s="12"/>
+      <c r="U38" s="12"/>
+      <c r="V38" s="12"/>
+      <c r="W38" s="12"/>
+      <c r="X38" s="12"/>
+    </row>
+    <row r="39" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" s="11"/>
+      <c r="L39" s="12"/>
+      <c r="U39" s="12"/>
+      <c r="V39" s="12"/>
+      <c r="W39" s="12"/>
+      <c r="X39" s="12"/>
+    </row>
+    <row r="40" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="L40" s="12"/>
+      <c r="U40" s="12"/>
+      <c r="V40" s="12"/>
+      <c r="W40" s="12"/>
+      <c r="X40" s="12"/>
+    </row>
+    <row r="41" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41" s="11"/>
+      <c r="L41" s="12"/>
+      <c r="U41" s="12"/>
+      <c r="V41" s="12"/>
+      <c r="W41" s="12"/>
+      <c r="X41" s="12"/>
+    </row>
+    <row r="42" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A42" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="L42" s="12"/>
+      <c r="U42" s="12"/>
+      <c r="V42" s="12"/>
+      <c r="W42" s="12"/>
+      <c r="X42" s="12"/>
+    </row>
+    <row r="43" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A43" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B43" s="11"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="L43" s="12"/>
+      <c r="U43" s="12"/>
+      <c r="V43" s="12"/>
+      <c r="W43" s="12"/>
+      <c r="X43" s="12"/>
+    </row>
+    <row r="44" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A44" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B44" s="11"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="L44" s="12"/>
+      <c r="U44" s="12"/>
+      <c r="V44" s="12"/>
+      <c r="W44" s="12"/>
+      <c r="X44" s="12"/>
+    </row>
+    <row r="45" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A45" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B45" s="11"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+      <c r="L45" s="12"/>
+      <c r="U45" s="12"/>
+      <c r="V45" s="12"/>
+      <c r="W45" s="12"/>
+      <c r="X45" s="12"/>
+    </row>
+    <row r="46" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" s="11"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="L46" s="12"/>
+      <c r="U46" s="12"/>
+      <c r="V46" s="12"/>
+      <c r="W46" s="12"/>
+      <c r="X46" s="12"/>
+    </row>
+    <row r="47" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="11"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+      <c r="L47" s="12"/>
+      <c r="U47" s="12"/>
+      <c r="V47" s="12"/>
+      <c r="W47" s="12"/>
+      <c r="X47" s="12"/>
+    </row>
+    <row r="48" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A48" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" s="11"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+      <c r="L48" s="12"/>
+      <c r="U48" s="12"/>
+      <c r="V48" s="12"/>
+      <c r="W48" s="12"/>
+      <c r="X48" s="12"/>
+    </row>
+    <row r="49" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A49" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" s="11"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+      <c r="L49" s="12"/>
+      <c r="U49" s="12"/>
+      <c r="V49" s="12"/>
+      <c r="W49" s="12"/>
+      <c r="X49" s="12"/>
+    </row>
+    <row r="50" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A50" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B50" s="11"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+      <c r="L50" s="12"/>
+      <c r="U50" s="12"/>
+      <c r="V50" s="12"/>
+      <c r="W50" s="12"/>
+      <c r="X50" s="12"/>
+    </row>
+    <row r="51" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A51" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="11"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+      <c r="L51" s="12"/>
+      <c r="U51" s="12"/>
+      <c r="V51" s="12"/>
+      <c r="W51" s="12"/>
+      <c r="X51" s="12"/>
+    </row>
+    <row r="52" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A52" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52" s="11"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
+      <c r="L52" s="12"/>
+      <c r="U52" s="12"/>
+      <c r="V52" s="12"/>
+      <c r="W52" s="12"/>
+      <c r="X52" s="12"/>
+    </row>
+    <row r="53" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A53" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B53" s="11"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="L53" s="12"/>
+      <c r="U53" s="12"/>
+      <c r="V53" s="12"/>
+      <c r="W53" s="12"/>
+      <c r="X53" s="12"/>
+    </row>
+    <row r="54" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A54" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" s="11"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="L54" s="12"/>
+      <c r="U54" s="12"/>
+      <c r="V54" s="12"/>
+      <c r="W54" s="12"/>
+      <c r="X54" s="12"/>
+    </row>
+    <row r="55" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A55" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55" s="11"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="L55" s="12"/>
+      <c r="U55" s="12"/>
+      <c r="V55" s="12"/>
+      <c r="W55" s="12"/>
+      <c r="X55" s="12"/>
+    </row>
+    <row r="56" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A56" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="L56" s="12"/>
+      <c r="U56" s="12"/>
+      <c r="V56" s="12"/>
+      <c r="W56" s="12"/>
+      <c r="X56" s="12"/>
+    </row>
+    <row r="57" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A57" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B57" s="11"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+      <c r="L57" s="12"/>
+      <c r="U57" s="12"/>
+      <c r="V57" s="12"/>
+      <c r="W57" s="12"/>
+      <c r="X57" s="12"/>
+    </row>
+    <row r="58" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A58" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B58" s="11"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+      <c r="L58" s="12"/>
+      <c r="U58" s="12"/>
+      <c r="V58" s="12"/>
+      <c r="W58" s="12"/>
+      <c r="X58" s="12"/>
+    </row>
+    <row r="59" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A59" s="26"/>
+      <c r="B59" s="27"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="L59" s="12"/>
+      <c r="U59" s="12"/>
+      <c r="V59" s="12"/>
+      <c r="W59" s="12"/>
+      <c r="X59" s="12"/>
+    </row>
+    <row r="60" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A60" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B60" s="7"/>
+      <c r="U60" s="12"/>
+      <c r="V60" s="12"/>
+    </row>
+    <row r="61" spans="1:24" ht="15.05" x14ac:dyDescent="0.25">
+      <c r="A61" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B61" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C61" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="D61" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E61" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F61" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G61" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="H61" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="U61" s="12"/>
+      <c r="V61" s="12"/>
+    </row>
+    <row r="62" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B62" s="2">
+        <v>100</v>
+      </c>
+      <c r="C62" s="28">
+        <v>820</v>
+      </c>
+      <c r="D62" s="28">
+        <v>827.69699099363697</v>
+      </c>
+      <c r="E62" s="3">
+        <f>D62/C62-1</f>
+        <v>9.3865743824841363E-3</v>
+      </c>
+      <c r="F62" s="5">
+        <f>3.16/1000</f>
+        <v>3.16E-3</v>
+      </c>
+      <c r="G62" s="1">
+        <v>2000</v>
+      </c>
+      <c r="H62" s="6">
+        <f>F62 * G62</f>
+        <v>6.32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B63" s="1">
+        <v>150</v>
+      </c>
+      <c r="C63" s="28">
+        <v>3055.23</v>
+      </c>
+      <c r="D63" s="29">
+        <v>3176.3473615429598</v>
+      </c>
+      <c r="E63" s="3">
+        <f>D63/C63-1</f>
+        <v>3.9642632974591141E-2</v>
+      </c>
+      <c r="F63" s="4">
+        <f>8.8/1000</f>
+        <v>8.8000000000000005E-3</v>
+      </c>
+      <c r="G63" s="1">
+        <v>2000</v>
+      </c>
+      <c r="H63" s="6">
+        <f t="shared" ref="H63:H66" si="0">F63 * G63</f>
+        <v>17.600000000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B64" s="2">
+        <v>200</v>
+      </c>
+      <c r="C64" s="28">
+        <v>1395.85</v>
+      </c>
+      <c r="D64" s="28">
+        <v>1363.1950523400101</v>
+      </c>
+      <c r="E64" s="3">
+        <f>D64/C64-1</f>
+        <v>-2.3394310033305721E-2</v>
+      </c>
+      <c r="F64" s="4">
+        <f>13.07/1000</f>
+        <v>1.307E-2</v>
+      </c>
+      <c r="G64" s="1">
+        <v>2000</v>
+      </c>
+      <c r="H64" s="6">
+        <f t="shared" si="0"/>
+        <v>26.14</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B65" s="1">
+        <v>250</v>
+      </c>
+      <c r="C65" s="28">
+        <v>38684</v>
+      </c>
+      <c r="D65" s="28">
+        <v>42104.2256917017</v>
+      </c>
+      <c r="E65" s="3">
+        <f>D65/C65-1</f>
+        <v>8.8414478639791572E-2</v>
+      </c>
+      <c r="F65" s="4">
+        <f>18.63/1000</f>
+        <v>1.8630000000000001E-2</v>
+      </c>
+      <c r="G65" s="1">
+        <v>3000</v>
+      </c>
+      <c r="H65" s="6">
+        <f t="shared" si="0"/>
+        <v>55.89</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B66" s="7">
+        <v>302</v>
+      </c>
+      <c r="C66" s="30">
+        <v>21736</v>
+      </c>
+      <c r="D66" s="29">
+        <v>22685.325526915502</v>
+      </c>
+      <c r="E66" s="3">
+        <f>D66/C66-1</f>
+        <v>4.367526347605355E-2</v>
+      </c>
+      <c r="F66" s="4">
+        <f>27.5/1000</f>
+        <v>2.75E-2</v>
+      </c>
+      <c r="G66" s="1">
+        <v>4000</v>
+      </c>
+      <c r="H66" s="1">
+        <f t="shared" si="0"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B67" s="7"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B68" s="7"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B69" s="7"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B70" s="7"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B71" s="7"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B72" s="7"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B73" s="7"/>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B74" s="7"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B75" s="7"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B76" s="7"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B77" s="7"/>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B78" s="7"/>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B79" s="7"/>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B80" s="7"/>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B81" s="7"/>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B82" s="7"/>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B83" s="7"/>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B84" s="7"/>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B85" s="7"/>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B86" s="7"/>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B87" s="7"/>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B88" s="7"/>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B89" s="7"/>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B90" s="7"/>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B91" s="7"/>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B92" s="7"/>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B93" s="7"/>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B94" s="7"/>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B95" s="7"/>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B96" s="7"/>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B97" s="7"/>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B98" s="7"/>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B99" s="7"/>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B100" s="7"/>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B101" s="7"/>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B102" s="7"/>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B103" s="7"/>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B104" s="7"/>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B105" s="7"/>
+    </row>
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B106" s="7"/>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B107" s="7"/>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B108" s="7"/>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B109" s="7"/>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B110" s="7"/>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B111" s="7"/>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B112" s="7"/>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B113" s="7"/>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B114" s="7"/>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B115" s="7"/>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B116" s="7"/>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B117" s="7"/>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B118" s="7"/>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B119" s="7"/>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B120" s="7"/>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B121" s="7"/>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B122" s="7"/>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B123" s="7"/>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B124" s="7"/>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B125" s="7"/>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B126" s="7"/>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B127" s="7"/>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B128" s="7"/>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B129" s="7"/>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B130" s="7"/>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B131" s="7"/>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B132" s="7"/>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B133" s="7"/>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B134" s="7"/>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B135" s="7"/>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B136" s="7"/>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B137" s="7"/>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B138" s="7"/>
+    </row>
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B139" s="7"/>
+    </row>
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B140" s="7"/>
+    </row>
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B141" s="7"/>
+    </row>
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B142" s="7"/>
+    </row>
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B143" s="7"/>
+    </row>
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B144" s="7"/>
+    </row>
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B145" s="7"/>
+    </row>
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B146" s="7"/>
+    </row>
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B147" s="7"/>
+    </row>
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B148" s="7"/>
+    </row>
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B149" s="7"/>
+    </row>
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B150" s="7"/>
+    </row>
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B151" s="7"/>
+    </row>
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B152" s="7"/>
+    </row>
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B153" s="7"/>
+    </row>
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B154" s="7"/>
+    </row>
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B155" s="7"/>
+    </row>
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B156" s="7"/>
+    </row>
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B157" s="7"/>
+    </row>
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B158" s="7"/>
+    </row>
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B159" s="7"/>
+    </row>
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B160" s="7"/>
+    </row>
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B161" s="7"/>
+    </row>
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B162" s="7"/>
+    </row>
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B163" s="7"/>
+    </row>
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B164" s="7"/>
+    </row>
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B165" s="7"/>
+    </row>
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B166" s="7"/>
+    </row>
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B167" s="7"/>
+    </row>
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B168" s="7"/>
+    </row>
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B169" s="7"/>
+    </row>
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B170" s="7"/>
+    </row>
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B171" s="7"/>
+    </row>
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B172" s="7"/>
+    </row>
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B173" s="7"/>
+    </row>
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B174" s="7"/>
+    </row>
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B175" s="7"/>
+    </row>
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B176" s="7"/>
+    </row>
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B177" s="7"/>
+    </row>
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B178" s="7"/>
+    </row>
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B179" s="7"/>
+    </row>
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B180" s="7"/>
+    </row>
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B181" s="7"/>
+    </row>
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B182" s="7"/>
+    </row>
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B183" s="7"/>
+    </row>
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B184" s="7"/>
+    </row>
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+    </row>
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B186" s="7"/>
+    </row>
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+    </row>
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+    </row>
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B189" s="7"/>
+    </row>
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B190" s="7"/>
+    </row>
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B191" s="7"/>
+    </row>
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B192" s="7"/>
+    </row>
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B193" s="7"/>
+    </row>
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B194" s="7"/>
+    </row>
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B195" s="7"/>
+    </row>
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B196" s="7"/>
+    </row>
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B197" s="7"/>
+    </row>
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B198" s="7"/>
+    </row>
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B199" s="7"/>
+    </row>
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B200" s="7"/>
+    </row>
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B201" s="7"/>
+    </row>
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B202" s="7"/>
+    </row>
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B203" s="7"/>
+    </row>
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B204" s="7"/>
+    </row>
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B205" s="7"/>
+    </row>
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B206" s="7"/>
+    </row>
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B207" s="7"/>
+    </row>
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B208" s="7"/>
+    </row>
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B209" s="7"/>
+    </row>
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B210" s="7"/>
+    </row>
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B211" s="7"/>
+    </row>
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B212" s="7"/>
+    </row>
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B213" s="7"/>
+    </row>
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B214" s="7"/>
+    </row>
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B215" s="7"/>
+    </row>
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B216" s="7"/>
+    </row>
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B217" s="7"/>
+    </row>
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B218" s="7"/>
+    </row>
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B219" s="7"/>
+    </row>
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B220" s="7"/>
+    </row>
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B221" s="7"/>
+    </row>
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B222" s="7"/>
+    </row>
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B223" s="7"/>
+    </row>
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B224" s="7"/>
+    </row>
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B225" s="7"/>
+    </row>
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B226" s="7"/>
+    </row>
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B227" s="7"/>
+    </row>
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B228" s="7"/>
+    </row>
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B229" s="7"/>
+    </row>
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B230" s="7"/>
+    </row>
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B231" s="7"/>
+    </row>
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B232" s="7"/>
+    </row>
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B233" s="7"/>
+    </row>
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B234" s="7"/>
+    </row>
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B235" s="7"/>
+    </row>
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B236" s="7"/>
+    </row>
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B237" s="7"/>
+    </row>
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B238" s="7"/>
+    </row>
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B239" s="7"/>
+    </row>
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B240" s="7"/>
+    </row>
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B241" s="7"/>
+    </row>
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B242" s="7"/>
+    </row>
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B243" s="7"/>
+    </row>
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B244" s="7"/>
+    </row>
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B245" s="7"/>
+    </row>
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B246" s="7"/>
+    </row>
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B247" s="7"/>
+    </row>
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B248" s="7"/>
+    </row>
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B249" s="7"/>
+    </row>
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B250" s="7"/>
+    </row>
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B251" s="7"/>
+    </row>
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B252" s="7"/>
+    </row>
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B253" s="7"/>
+    </row>
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B254" s="7"/>
+    </row>
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B255" s="7"/>
+    </row>
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B256" s="7"/>
+    </row>
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B257" s="7"/>
+    </row>
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B258" s="7"/>
+    </row>
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B259" s="7"/>
+    </row>
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B260" s="7"/>
+    </row>
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B261" s="7"/>
+    </row>
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B262" s="7"/>
+    </row>
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B263" s="7"/>
+    </row>
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B264" s="7"/>
+    </row>
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B265" s="7"/>
+    </row>
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B266" s="7"/>
+    </row>
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B267" s="7"/>
+    </row>
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B268" s="7"/>
+    </row>
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B269" s="7"/>
+    </row>
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B270" s="7"/>
+    </row>
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B271" s="7"/>
+    </row>
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B272" s="7"/>
+    </row>
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B273" s="7"/>
+    </row>
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B274" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X280"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.15" x14ac:dyDescent="0.25"/>
@@ -801,7 +2394,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.05" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="16"/>
@@ -965,7 +2558,7 @@
     </row>
     <row r="20" spans="1:24" s="9" customFormat="1" ht="12.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="B20" s="11"/>
       <c r="L20" s="12"/>
@@ -1713,15 +3306,15 @@
         <v>-1.6412392354492322E-3</v>
       </c>
       <c r="F65" s="5">
-        <f>4.79/1000</f>
-        <v>4.79E-3</v>
+        <f>4.77/1000</f>
+        <v>4.7699999999999999E-3</v>
       </c>
       <c r="G65" s="1">
         <v>2000</v>
       </c>
       <c r="H65" s="6">
         <f>F65 * G65</f>
-        <v>9.58</v>
+        <v>9.5399999999999991</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
@@ -1742,15 +3335,15 @@
         <v>-4.4820130025886917E-2</v>
       </c>
       <c r="F66" s="4">
-        <f>12.42/1000</f>
-        <v>1.242E-2</v>
+        <f>12.27/1000</f>
+        <v>1.227E-2</v>
       </c>
       <c r="G66" s="1">
         <v>2000</v>
       </c>
       <c r="H66" s="6">
         <f t="shared" ref="H66:H70" si="1">F66 * G66</f>
-        <v>24.84</v>
+        <v>24.54</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
@@ -1771,15 +3364,15 @@
         <v>-3.7795953302666163E-6</v>
       </c>
       <c r="F67" s="4">
-        <f>6.65/1000</f>
-        <v>6.6500000000000005E-3</v>
+        <f>6.41/1000</f>
+        <v>6.4099999999999999E-3</v>
       </c>
       <c r="G67" s="1">
         <v>2000</v>
       </c>
       <c r="H67" s="6">
         <f t="shared" si="1"/>
-        <v>13.3</v>
+        <v>12.82</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -1800,15 +3393,15 @@
         <v>-5.8207641997487514E-6</v>
       </c>
       <c r="F68" s="4">
-        <f>22.92/1000</f>
-        <v>2.2920000000000003E-2</v>
+        <f>22.76/1000</f>
+        <v>2.2760000000000002E-2</v>
       </c>
       <c r="G68" s="1">
         <v>2000</v>
       </c>
       <c r="H68" s="6">
         <f t="shared" si="1"/>
-        <v>45.84</v>
+        <v>45.52</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -1829,15 +3422,15 @@
         <v>-1.57441856144237E-2</v>
       </c>
       <c r="F69" s="4">
-        <f>12.69/1000</f>
-        <v>1.269E-2</v>
+        <f>5.4/1000</f>
+        <v>5.4000000000000003E-3</v>
       </c>
       <c r="G69" s="1">
         <v>2000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="1"/>
-        <v>25.38</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -1858,15 +3451,15 @@
         <v>-7.7474249471089163E-2</v>
       </c>
       <c r="F70" s="4">
-        <f>5.25/1000</f>
-        <v>5.2500000000000003E-3</v>
+        <f>12.43/1000</f>
+        <v>1.243E-2</v>
       </c>
       <c r="G70" s="1">
         <v>2000</v>
       </c>
       <c r="H70" s="6">
         <f t="shared" si="1"/>
-        <v>10.5</v>
+        <v>24.86</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
add route slack time evaluation
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Academia\Research related\dev\VRP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB94505-E4A1-4643-9A20-E64ED73834C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD19221-6703-46B8-8CDC-7619359E026A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3251,15 +3251,15 @@
         <v>9.093610682541442E-3</v>
       </c>
       <c r="F67" s="5">
-        <f>4.27/1000</f>
-        <v>4.2699999999999995E-3</v>
+        <f>4.56/1000</f>
+        <v>4.5599999999999998E-3</v>
       </c>
       <c r="G67" s="1">
         <v>5000</v>
       </c>
       <c r="H67" s="6">
         <f>F67 * G67</f>
-        <v>21.349999999999998</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
@@ -3280,15 +3280,15 @@
         <v>-6.0416154308814418E-2</v>
       </c>
       <c r="F68" s="4">
-        <f>10.79/1000</f>
-        <v>1.0789999999999999E-2</v>
+        <f>11.92/1000</f>
+        <v>1.192E-2</v>
       </c>
       <c r="G68" s="1">
         <v>5000</v>
       </c>
       <c r="H68" s="6">
         <f t="shared" ref="H68:H72" si="1">F68 * G68</f>
-        <v>53.949999999999996</v>
+        <v>59.6</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
@@ -3309,15 +3309,15 @@
         <v>-3.7795946365992705E-6</v>
       </c>
       <c r="F69" s="4">
-        <f>5.16/1000</f>
-        <v>5.1600000000000005E-3</v>
+        <f>5.58/1000</f>
+        <v>5.5799999999999999E-3</v>
       </c>
       <c r="G69" s="1">
         <v>5000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="1"/>
-        <v>25.800000000000004</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -3338,15 +3338,15 @@
         <v>-5.8207599751280981E-6</v>
       </c>
       <c r="F70" s="4">
-        <f>18.95/1000</f>
-        <v>1.8949999999999998E-2</v>
+        <f>19.71/1000</f>
+        <v>1.9710000000000002E-2</v>
       </c>
       <c r="G70" s="1">
         <v>5000</v>
       </c>
       <c r="H70" s="6">
         <f t="shared" si="1"/>
-        <v>94.749999999999986</v>
+        <v>98.550000000000011</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
@@ -3367,15 +3367,15 @@
         <v>-2.7544773361226738E-2</v>
       </c>
       <c r="F71" s="4">
-        <f>4.52/1000</f>
-        <v>4.5199999999999997E-3</v>
+        <f>4.82/1000</f>
+        <v>4.8200000000000005E-3</v>
       </c>
       <c r="G71" s="1">
         <v>5000</v>
       </c>
       <c r="H71" s="6">
         <f t="shared" si="1"/>
-        <v>22.599999999999998</v>
+        <v>24.1</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
@@ -3396,15 +3396,15 @@
         <v>-8.4777320115295263E-2</v>
       </c>
       <c r="F72" s="4">
-        <f>9.57/1000</f>
-        <v>9.5700000000000004E-3</v>
+        <f>11.12/1000</f>
+        <v>1.112E-2</v>
       </c>
       <c r="G72" s="1">
         <v>5000</v>
       </c>
       <c r="H72" s="6">
         <f t="shared" si="1"/>
-        <v>47.85</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
combine inter intra opt
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Academia\Research related\dev\VRP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BE13049-74F5-4BEC-89FA-3D26049DE89E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8CCF451-8549-46EE-AC6C-075C71C1ACEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VRP Benchmarking" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="89">
   <si>
     <t>Best known</t>
   </si>
@@ -227,12 +227,6 @@
     <t>                    :regret3!</t>
   </si>
   <si>
-    <t>                    :intraopt!      ,</t>
-  </si>
-  <si>
-    <t>                    :interopt!      ,</t>
-  </si>
-  <si>
     <t>                    :split!         ,</t>
   </si>
   <si>
@@ -303,6 +297,12 @@
   </si>
   <si>
     <t>        𝜃   =   0.9975                 ,</t>
+  </si>
+  <si>
+    <t>                    :opt!           ,</t>
+  </si>
+  <si>
+    <t>                    :opt!           ,</t>
   </si>
 </sst>
 </file>
@@ -816,7 +816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EB48D86-1312-4781-AFB7-1DCAC26244E4}">
-  <dimension ref="A1:X276"/>
+  <dimension ref="A1:X275"/>
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" style="1" customWidth="1"/>
@@ -832,7 +832,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="16"/>
@@ -951,16 +951,16 @@
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:6" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -994,7 +994,7 @@
     </row>
     <row r="19" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B19" s="12"/>
       <c r="W19" s="12"/>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="20" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B20" s="12"/>
       <c r="W20" s="12"/>
@@ -1010,7 +1010,7 @@
     </row>
     <row r="21" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B21" s="12"/>
       <c r="U21" s="12"/>
@@ -1184,7 +1184,7 @@
     </row>
     <row r="38" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12"/>
@@ -1201,7 +1201,7 @@
     </row>
     <row r="39" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="12"/>
@@ -1218,7 +1218,7 @@
     </row>
     <row r="40" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="12"/>
@@ -1235,7 +1235,7 @@
     </row>
     <row r="41" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="12"/>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="47" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A47" s="12" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="B47" s="12"/>
       <c r="H47" s="9"/>
@@ -1330,7 +1330,7 @@
     </row>
     <row r="48" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A48" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B48" s="12"/>
       <c r="H48" s="9"/>
@@ -1341,7 +1341,7 @@
     </row>
     <row r="49" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A49" s="12" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="B49" s="12"/>
       <c r="H49" s="9"/>
@@ -1352,7 +1352,7 @@
     </row>
     <row r="50" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B50" s="12"/>
       <c r="H50" s="9"/>
@@ -1363,7 +1363,7 @@
     </row>
     <row r="51" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
-        <v>7</v>
+        <v>74</v>
       </c>
       <c r="B51" s="12"/>
       <c r="H51" s="9"/>
@@ -1374,7 +1374,7 @@
     </row>
     <row r="52" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A52" s="12" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B52" s="12"/>
       <c r="H52" s="9"/>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="53" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B53" s="12"/>
       <c r="H53" s="9"/>
@@ -1396,10 +1396,9 @@
     </row>
     <row r="54" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A54" s="12" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="B54" s="12"/>
-      <c r="H54" s="9"/>
       <c r="U54" s="12"/>
       <c r="V54" s="12"/>
       <c r="W54" s="12"/>
@@ -1407,7 +1406,7 @@
     </row>
     <row r="55" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A55" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B55" s="12"/>
       <c r="U55" s="12"/>
@@ -1417,7 +1416,7 @@
     </row>
     <row r="56" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A56" s="12" t="s">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="B56" s="12"/>
       <c r="U56" s="12"/>
@@ -1427,7 +1426,7 @@
     </row>
     <row r="57" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A57" s="12" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B57" s="12"/>
       <c r="U57" s="12"/>
@@ -1437,7 +1436,7 @@
     </row>
     <row r="58" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A58" s="12" t="s">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="B58" s="12"/>
       <c r="U58" s="12"/>
@@ -1447,7 +1446,7 @@
     </row>
     <row r="59" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A59" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B59" s="12"/>
       <c r="U59" s="12"/>
@@ -1457,7 +1456,7 @@
     </row>
     <row r="60" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A60" s="12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B60" s="12"/>
       <c r="U60" s="12"/>
@@ -1467,204 +1466,197 @@
     </row>
     <row r="61" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A61" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B61" s="12"/>
+        <v>64</v>
+      </c>
       <c r="U61" s="12"/>
       <c r="V61" s="12"/>
-      <c r="W61" s="12"/>
-      <c r="X61" s="12"/>
     </row>
     <row r="62" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A62" s="12" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="U62" s="12"/>
       <c r="V62" s="12"/>
     </row>
-    <row r="63" spans="1:24" ht="14" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="U63" s="12"/>
-      <c r="V63" s="12"/>
+    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A64" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B64" s="7"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A65" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B65" s="7"/>
+      <c r="A65" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="D65" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E65" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F65" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G65" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="H65" s="18" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B66" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="C66" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="D66" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="E66" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="F66" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="G66" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H66" s="18" t="s">
-        <v>5</v>
+      <c r="A66" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B66" s="2">
+        <v>100</v>
+      </c>
+      <c r="C66" s="25">
+        <v>820</v>
+      </c>
+      <c r="D66" s="25">
+        <v>819.55754418732204</v>
+      </c>
+      <c r="E66" s="3">
+        <f>D66/C66-1</f>
+        <v>-5.3958025936340359E-4</v>
+      </c>
+      <c r="F66" s="5">
+        <f>3.02/1000</f>
+        <v>3.0200000000000001E-3</v>
+      </c>
+      <c r="G66" s="1">
+        <v>5000</v>
+      </c>
+      <c r="H66" s="6">
+        <f>F66 * G66</f>
+        <v>15.100000000000001</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B67" s="2">
-        <v>100</v>
+      <c r="A67" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B67" s="1">
+        <v>150</v>
       </c>
       <c r="C67" s="25">
-        <v>820</v>
-      </c>
-      <c r="D67" s="25">
-        <v>819.55754418737604</v>
+        <v>3055.23</v>
+      </c>
+      <c r="D67" s="26">
+        <v>3119.2520262377302</v>
       </c>
       <c r="E67" s="3">
         <f>D67/C67-1</f>
-        <v>-5.3958025929756737E-4</v>
-      </c>
-      <c r="F67" s="5">
-        <f>3.3/1000</f>
-        <v>3.3E-3</v>
+        <v>2.0954895781243987E-2</v>
+      </c>
+      <c r="F67" s="4">
+        <f>8.38/1000</f>
+        <v>8.3800000000000003E-3</v>
       </c>
       <c r="G67" s="1">
         <v>5000</v>
       </c>
       <c r="H67" s="6">
-        <f>F67 * G67</f>
-        <v>16.5</v>
+        <f t="shared" ref="H67:H70" si="0">F67 * G67</f>
+        <v>41.9</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B68" s="1">
-        <v>150</v>
+      <c r="A68" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B68" s="2">
+        <v>200</v>
       </c>
       <c r="C68" s="25">
-        <v>3055.23</v>
-      </c>
-      <c r="D68" s="26">
-        <v>3104.0276306494802</v>
+        <v>1395.85</v>
+      </c>
+      <c r="D68" s="25">
+        <v>1333.4754040789301</v>
       </c>
       <c r="E68" s="3">
         <f>D68/C68-1</f>
-        <v>1.5971835393564504E-2</v>
+        <v>-4.4685744113672543E-2</v>
       </c>
       <c r="F68" s="4">
-        <f>8.42/1000</f>
-        <v>8.4200000000000004E-3</v>
+        <f>11.13/1000</f>
+        <v>1.1130000000000001E-2</v>
       </c>
       <c r="G68" s="1">
         <v>5000</v>
       </c>
       <c r="H68" s="6">
-        <f t="shared" ref="H68:H71" si="0">F68 * G68</f>
-        <v>42.1</v>
+        <f t="shared" si="0"/>
+        <v>55.650000000000006</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A69" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B69" s="2">
-        <v>200</v>
+      <c r="A69" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B69" s="1">
+        <v>250</v>
       </c>
       <c r="C69" s="25">
-        <v>1395.85</v>
+        <v>38684</v>
       </c>
       <c r="D69" s="25">
-        <v>1333.4039064419301</v>
+        <v>41023.472215590598</v>
       </c>
       <c r="E69" s="3">
         <f>D69/C69-1</f>
-        <v>-4.4736965689773145E-2</v>
+        <v>6.0476481635575396E-2</v>
       </c>
       <c r="F69" s="4">
-        <f>11.23/1000</f>
-        <v>1.123E-2</v>
+        <f>16.54/1000</f>
+        <v>1.6539999999999999E-2</v>
       </c>
       <c r="G69" s="1">
         <v>5000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="0"/>
-        <v>56.15</v>
+        <v>82.699999999999989</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B70" s="1">
-        <v>250</v>
-      </c>
-      <c r="C70" s="25">
-        <v>38684</v>
-      </c>
-      <c r="D70" s="25">
-        <v>40964.220637907703</v>
+        <v>73</v>
+      </c>
+      <c r="B70" s="7">
+        <v>302</v>
+      </c>
+      <c r="C70" s="27">
+        <v>21736</v>
+      </c>
+      <c r="D70" s="26">
+        <v>22858.740516695099</v>
       </c>
       <c r="E70" s="3">
         <f>D70/C70-1</f>
-        <v>5.8944799863191566E-2</v>
+        <v>5.1653501872244156E-2</v>
       </c>
       <c r="F70" s="4">
-        <f>15.91/1000</f>
-        <v>1.5910000000000001E-2</v>
+        <f>21.31/1000</f>
+        <v>2.1309999999999999E-2</v>
       </c>
       <c r="G70" s="1">
         <v>5000</v>
       </c>
-      <c r="H70" s="6">
+      <c r="H70" s="1">
         <f t="shared" si="0"/>
-        <v>79.55</v>
+        <v>106.55</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B71" s="7">
-        <v>302</v>
-      </c>
-      <c r="C71" s="27">
-        <v>21736</v>
-      </c>
-      <c r="D71" s="26">
-        <v>22753.471385720899</v>
-      </c>
-      <c r="E71" s="3">
-        <f>D71/C71-1</f>
-        <v>4.6810424444281296E-2</v>
-      </c>
-      <c r="F71" s="4">
-        <f>20.91/1000</f>
-        <v>2.0910000000000002E-2</v>
-      </c>
-      <c r="G71" s="1">
-        <v>5000</v>
-      </c>
-      <c r="H71" s="1">
-        <f t="shared" si="0"/>
-        <v>104.55000000000001</v>
-      </c>
+      <c r="B71" s="7"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B72" s="7"/>
@@ -2277,9 +2269,6 @@
     </row>
     <row r="275" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B275" s="7"/>
-    </row>
-    <row r="276" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B276" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2289,7 +2278,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X282"/>
+  <dimension ref="A1:X281"/>
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" style="1" customWidth="1"/>
@@ -2305,7 +2294,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="16"/>
@@ -2424,7 +2413,7 @@
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D15" s="1"/>
     </row>
@@ -2433,7 +2422,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2460,7 +2449,7 @@
     </row>
     <row r="19" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B19" s="11"/>
       <c r="L19" s="12"/>
@@ -2469,7 +2458,7 @@
     </row>
     <row r="20" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B20" s="11"/>
       <c r="L20" s="12"/>
@@ -2478,7 +2467,7 @@
     </row>
     <row r="21" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -2767,7 +2756,7 @@
     </row>
     <row r="38" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12"/>
@@ -2784,7 +2773,7 @@
     </row>
     <row r="39" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="12"/>
@@ -2801,7 +2790,7 @@
     </row>
     <row r="40" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="12"/>
@@ -2818,7 +2807,7 @@
     </row>
     <row r="41" spans="1:24" s="9" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="12"/>
@@ -2920,7 +2909,7 @@
     </row>
     <row r="47" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A47" s="12" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="B47" s="12"/>
       <c r="C47" s="12"/>
@@ -2937,7 +2926,7 @@
     </row>
     <row r="48" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A48" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="12"/>
@@ -2954,7 +2943,7 @@
     </row>
     <row r="49" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A49" s="12" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="B49" s="12"/>
       <c r="C49" s="12"/>
@@ -2971,7 +2960,7 @@
     </row>
     <row r="50" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="12"/>
@@ -2988,7 +2977,7 @@
     </row>
     <row r="51" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
-        <v>7</v>
+        <v>74</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="12"/>
@@ -3005,7 +2994,7 @@
     </row>
     <row r="52" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A52" s="12" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="12"/>
@@ -3022,7 +3011,7 @@
     </row>
     <row r="53" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B53" s="12"/>
       <c r="C53" s="12"/>
@@ -3039,7 +3028,7 @@
     </row>
     <row r="54" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A54" s="12" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="B54" s="12"/>
       <c r="C54" s="12"/>
@@ -3056,7 +3045,7 @@
     </row>
     <row r="55" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A55" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="12"/>
@@ -3073,7 +3062,7 @@
     </row>
     <row r="56" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A56" s="12" t="s">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="B56" s="12"/>
       <c r="C56" s="12"/>
@@ -3090,7 +3079,7 @@
     </row>
     <row r="57" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A57" s="12" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="12"/>
@@ -3107,7 +3096,7 @@
     </row>
     <row r="58" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A58" s="12" t="s">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="B58" s="12"/>
       <c r="C58" s="12"/>
@@ -3124,7 +3113,7 @@
     </row>
     <row r="59" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A59" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="12"/>
@@ -3141,7 +3130,7 @@
     </row>
     <row r="60" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A60" s="12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B60" s="12"/>
       <c r="C60" s="12"/>
@@ -3158,7 +3147,7 @@
     </row>
     <row r="61" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A61" s="12" t="s">
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="12"/>
@@ -3167,15 +3156,12 @@
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
       <c r="H61" s="12"/>
-      <c r="L61" s="12"/>
       <c r="U61" s="12"/>
       <c r="V61" s="12"/>
-      <c r="W61" s="12"/>
-      <c r="X61" s="12"/>
     </row>
     <row r="62" spans="1:24" ht="14" x14ac:dyDescent="0.3">
       <c r="A62" s="12" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="B62" s="12"/>
       <c r="C62" s="12"/>
@@ -3187,225 +3173,214 @@
       <c r="U62" s="12"/>
       <c r="V62" s="12"/>
     </row>
-    <row r="63" spans="1:24" ht="14" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B63" s="12"/>
-      <c r="C63" s="12"/>
-      <c r="D63" s="12"/>
-      <c r="E63" s="12"/>
-      <c r="F63" s="12"/>
-      <c r="G63" s="12"/>
-      <c r="H63" s="12"/>
-      <c r="U63" s="12"/>
-      <c r="V63" s="12"/>
+    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A64" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B64" s="7"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A65" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B65" s="7"/>
+      <c r="A65" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="D65" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E65" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F65" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G65" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="H65" s="18" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B66" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="C66" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="D66" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="E66" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="F66" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="G66" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H66" s="18" t="s">
-        <v>5</v>
+      <c r="A66" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B66" s="2">
+        <v>100</v>
+      </c>
+      <c r="C66" s="6">
+        <v>1645.79</v>
+      </c>
+      <c r="D66" s="6">
+        <v>1644.7048641157</v>
+      </c>
+      <c r="E66" s="3">
+        <f>D66/C66-1</f>
+        <v>-6.5934042879101096E-4</v>
+      </c>
+      <c r="F66" s="5">
+        <f>5.14/1000</f>
+        <v>5.1399999999999996E-3</v>
+      </c>
+      <c r="G66" s="1">
+        <v>5000</v>
+      </c>
+      <c r="H66" s="6">
+        <f>F66 * G66</f>
+        <v>25.7</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
-        <v>41</v>
+      <c r="A67" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="B67" s="2">
         <v>100</v>
       </c>
-      <c r="C67" s="6">
-        <v>1645.79</v>
-      </c>
-      <c r="D67" s="6">
-        <v>1649.0599551073999</v>
+      <c r="C67" s="24">
+        <v>1252.3699999999999</v>
+      </c>
+      <c r="D67" s="24">
+        <v>1179.9333546359801</v>
       </c>
       <c r="E67" s="3">
-        <f>D67/C67-1</f>
-        <v>1.9868604787973698E-3</v>
-      </c>
-      <c r="F67" s="5">
-        <f>5.17/1000</f>
-        <v>5.1700000000000001E-3</v>
+        <f t="shared" ref="E67:E71" si="0">D67/C67-1</f>
+        <v>-5.7839652310435308E-2</v>
+      </c>
+      <c r="F67" s="4">
+        <f>13.49/1000</f>
+        <v>1.349E-2</v>
       </c>
       <c r="G67" s="1">
         <v>5000</v>
       </c>
       <c r="H67" s="6">
-        <f>F67 * G67</f>
-        <v>25.85</v>
+        <f t="shared" ref="H67:H71" si="1">F67 * G67</f>
+        <v>67.45</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
-        <v>42</v>
+      <c r="A68" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="B68" s="2">
         <v>100</v>
       </c>
-      <c r="C68" s="24">
-        <v>1252.3699999999999</v>
-      </c>
-      <c r="D68" s="24">
-        <v>1168.62258735657</v>
+      <c r="C68" s="6">
+        <v>828.94</v>
+      </c>
+      <c r="D68" s="6">
+        <v>828.936866942812</v>
       </c>
       <c r="E68" s="3">
-        <f t="shared" ref="E68:E72" si="0">D68/C68-1</f>
-        <v>-6.6871142428699182E-2</v>
+        <f t="shared" si="0"/>
+        <v>-3.7795946487007015E-6</v>
       </c>
       <c r="F68" s="4">
-        <f>12.48/1000</f>
-        <v>1.248E-2</v>
+        <f>5.85/1000</f>
+        <v>5.8499999999999993E-3</v>
       </c>
       <c r="G68" s="1">
         <v>5000</v>
       </c>
       <c r="H68" s="6">
-        <f t="shared" ref="H68:H72" si="1">F68 * G68</f>
-        <v>62.4</v>
+        <f t="shared" si="1"/>
+        <v>29.249999999999996</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B69" s="2">
         <v>100</v>
       </c>
       <c r="C69" s="6">
-        <v>828.94</v>
+        <v>591.55999999999995</v>
       </c>
       <c r="D69" s="6">
-        <v>828.936866942812</v>
+        <v>591.55655667143196</v>
       </c>
       <c r="E69" s="3">
         <f t="shared" si="0"/>
-        <v>-3.7795946487007015E-6</v>
+        <v>-5.8207596321802058E-6</v>
       </c>
       <c r="F69" s="4">
-        <f>6.05/1000</f>
-        <v>6.0499999999999998E-3</v>
+        <f>21.05/1000</f>
+        <v>2.1049999999999999E-2</v>
       </c>
       <c r="G69" s="1">
         <v>5000</v>
       </c>
       <c r="H69" s="6">
         <f t="shared" si="1"/>
-        <v>30.25</v>
+        <v>105.25</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B70" s="2">
         <v>100</v>
       </c>
       <c r="C70" s="6">
-        <v>591.55999999999995</v>
+        <v>1696.94</v>
       </c>
       <c r="D70" s="6">
-        <v>591.55655667143196</v>
+        <v>1645.5434971790201</v>
       </c>
       <c r="E70" s="3">
         <f t="shared" si="0"/>
-        <v>-5.8207596321802058E-6</v>
+        <v>-3.028775491235991E-2</v>
       </c>
       <c r="F70" s="4">
-        <f>21.02/1000</f>
-        <v>2.102E-2</v>
+        <f>5.04/1000</f>
+        <v>5.0400000000000002E-3</v>
       </c>
       <c r="G70" s="1">
         <v>5000</v>
       </c>
       <c r="H70" s="6">
         <f t="shared" si="1"/>
-        <v>105.10000000000001</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A71" s="2" t="s">
-        <v>45</v>
+      <c r="A71" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="B71" s="2">
         <v>100</v>
       </c>
-      <c r="C71" s="6">
-        <v>1696.94</v>
-      </c>
-      <c r="D71" s="6">
-        <v>1645.6655852073</v>
+      <c r="C71" s="24">
+        <v>1406.91</v>
+      </c>
+      <c r="D71" s="24">
+        <v>1310.38479266175</v>
       </c>
       <c r="E71" s="3">
         <f t="shared" si="0"/>
-        <v>-3.0215808922354426E-2</v>
+        <v>-6.8607947443866446E-2</v>
       </c>
       <c r="F71" s="4">
-        <f>5.31/1000</f>
-        <v>5.3099999999999996E-3</v>
+        <f>10.61/1000</f>
+        <v>1.061E-2</v>
       </c>
       <c r="G71" s="1">
         <v>5000</v>
       </c>
       <c r="H71" s="6">
         <f t="shared" si="1"/>
-        <v>26.549999999999997</v>
+        <v>53.05</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B72" s="2">
-        <v>100</v>
-      </c>
-      <c r="C72" s="24">
-        <v>1406.91</v>
-      </c>
-      <c r="D72" s="24">
-        <v>1287.7742416317201</v>
-      </c>
-      <c r="E72" s="3">
-        <f t="shared" si="0"/>
-        <v>-8.4679018820166152E-2</v>
-      </c>
-      <c r="F72" s="4">
-        <f>12.38/1000</f>
-        <v>1.238E-2</v>
-      </c>
-      <c r="G72" s="1">
-        <v>5000</v>
-      </c>
-      <c r="H72" s="6">
-        <f t="shared" si="1"/>
-        <v>61.9</v>
-      </c>
+      <c r="B72" s="7"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B73" s="7"/>
@@ -4033,9 +4008,6 @@
     </row>
     <row r="281" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B281" s="7"/>
-    </row>
-    <row r="282" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B282" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>